<commit_message>
Avant update model TK propre
</commit_message>
<xml_diff>
--- a/data/Data_TK_long.xlsx
+++ b/data/Data_TK_long.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lisagollot/Library/CloudStorage/OneDrive-Personnel/Documents/0_These/0_RepoGit/ew-mix-epximd/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lisagollot/Library/CloudStorage/OneDrive-Personnel/Documents/0_These/0_RepoGit/Ew-Mix-TK/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C79392C5-4E40-C74E-952B-84E969DC1EBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08B66484-EA08-C545-8CFE-7A854BCD00FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="-4080" windowWidth="38400" windowHeight="21100" xr2:uid="{63D67807-0DCA-1F4C-A29E-414A7CCA2C56}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{63D67807-0DCA-1F4C-A29E-414A7CCA2C56}"/>
   </bookViews>
   <sheets>
     <sheet name="TK" sheetId="2" r:id="rId1"/>
@@ -3229,7 +3229,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="54" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:17" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" s="6">
         <v>45439.629166666666</v>
       </c>
@@ -3275,7 +3275,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="55" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" s="16">
         <v>45439.629166666666</v>
       </c>
@@ -3730,7 +3730,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="65" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A65" s="7">
         <v>45439.636805555558</v>
       </c>
@@ -8621,7 +8621,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="182" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A182" s="8">
         <v>45460.625</v>
       </c>
@@ -8658,7 +8658,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="183" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A183" s="17">
         <v>45460.625</v>
       </c>
@@ -9028,7 +9028,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="193" spans="1:17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A193" s="9">
         <v>45460.625</v>
       </c>
@@ -9845,7 +9845,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="214" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A214" s="8">
         <v>45474.416666666664</v>
       </c>
@@ -9884,7 +9884,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="215" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A215" s="17">
         <v>45474.416666666664</v>
       </c>
@@ -10274,7 +10274,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="225" spans="1:17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A225" s="9">
         <v>45481.416666666664</v>
       </c>
@@ -16342,7 +16342,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="374" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="374" spans="1:17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A374" s="6">
         <v>45475.666666666664</v>
       </c>
@@ -16387,7 +16387,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="375" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="375" spans="1:17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A375" s="6">
         <v>45475.666666666664</v>
       </c>
@@ -16837,7 +16837,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="385" spans="1:17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="385" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A385" s="6">
         <v>45482.690972222219</v>
       </c>
@@ -19766,8 +19766,7 @@
   <autoFilter ref="A1:Q449" xr:uid="{AE06E5C9-F603-BD4A-AB05-F790F7B78C9A}">
     <filterColumn colId="6">
       <filters>
-        <filter val="105"/>
-        <filter val="106"/>
+        <filter val="124"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>